<commit_message>
chore(data-release): publish site data 2026-09-06 02:00:46 UTC
</commit_message>
<xml_diff>
--- a/diseases/d009/2026-2029.xlsx
+++ b/diseases/d009/2026-2029.xlsx
@@ -45207,13 +45207,13 @@
         </is>
       </c>
       <c r="N241" t="n">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="O241" t="n">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="R241" t="n">
-        <v>0.844954886773332</v>
+        <v>0.8430169168495401</v>
       </c>
       <c r="S241" t="inlineStr">
         <is>
@@ -46976,7 +46976,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>154370</v>
+        <v>154369</v>
       </c>
     </row>
     <row r="16">

</xml_diff>